<commit_message>
Updated UI, global client selection, 3CA and 3CB tax report templates
</commit_message>
<xml_diff>
--- a/clients/Abhishek/AY 2026-27/document_checklist.xlsx
+++ b/clients/Abhishek/AY 2026-27/document_checklist.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="111">
   <si>
     <t>Category</t>
   </si>
@@ -65,6 +65,9 @@
   </si>
   <si>
     <t>Final Audit Review Data</t>
+  </si>
+  <si>
+    <t>Balance Sheet Supporting Data</t>
   </si>
   <si>
     <t>Trial_Balance</t>
@@ -675,7 +678,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D130"/>
+  <dimension ref="A1:D143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -697,10 +700,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -708,10 +711,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -719,10 +722,10 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -730,10 +733,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -741,10 +744,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -752,10 +755,10 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -763,10 +766,10 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -774,10 +777,10 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -785,10 +788,10 @@
         <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -796,10 +799,10 @@
         <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -807,10 +810,10 @@
         <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -818,10 +821,10 @@
         <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -829,10 +832,10 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -840,10 +843,10 @@
         <v>5</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -851,10 +854,10 @@
         <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -862,10 +865,10 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -873,10 +876,10 @@
         <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -884,10 +887,10 @@
         <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -895,10 +898,10 @@
         <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C20" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -906,10 +909,10 @@
         <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C21" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -917,10 +920,10 @@
         <v>6</v>
       </c>
       <c r="B22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C22" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -928,10 +931,10 @@
         <v>6</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C23" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -939,10 +942,10 @@
         <v>6</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C24" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -950,10 +953,10 @@
         <v>6</v>
       </c>
       <c r="B25" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C25" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -961,10 +964,10 @@
         <v>6</v>
       </c>
       <c r="B26" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C26" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -972,10 +975,10 @@
         <v>7</v>
       </c>
       <c r="B27" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C27" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -983,10 +986,10 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C28" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -994,10 +997,10 @@
         <v>7</v>
       </c>
       <c r="B29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1005,10 +1008,10 @@
         <v>7</v>
       </c>
       <c r="B30" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C30" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1016,10 +1019,10 @@
         <v>7</v>
       </c>
       <c r="B31" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C31" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1027,10 +1030,10 @@
         <v>7</v>
       </c>
       <c r="B32" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C32" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1038,10 +1041,10 @@
         <v>7</v>
       </c>
       <c r="B33" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C33" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1049,10 +1052,10 @@
         <v>7</v>
       </c>
       <c r="B34" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C34" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1060,10 +1063,10 @@
         <v>7</v>
       </c>
       <c r="B35" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -1071,10 +1074,10 @@
         <v>7</v>
       </c>
       <c r="B36" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C36" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -1082,10 +1085,10 @@
         <v>7</v>
       </c>
       <c r="B37" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C37" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1093,10 +1096,10 @@
         <v>7</v>
       </c>
       <c r="B38" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C38" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -1104,10 +1107,10 @@
         <v>8</v>
       </c>
       <c r="B39" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C39" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -1115,10 +1118,10 @@
         <v>8</v>
       </c>
       <c r="B40" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C40" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -1126,10 +1129,10 @@
         <v>8</v>
       </c>
       <c r="B41" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C41" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -1137,10 +1140,10 @@
         <v>8</v>
       </c>
       <c r="B42" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C42" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -1148,10 +1151,10 @@
         <v>8</v>
       </c>
       <c r="B43" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C43" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -1159,10 +1162,10 @@
         <v>8</v>
       </c>
       <c r="B44" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C44" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -1170,10 +1173,10 @@
         <v>8</v>
       </c>
       <c r="B45" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C45" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -1181,10 +1184,10 @@
         <v>8</v>
       </c>
       <c r="B46" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C46" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -1192,10 +1195,10 @@
         <v>8</v>
       </c>
       <c r="B47" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C47" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -1203,10 +1206,10 @@
         <v>8</v>
       </c>
       <c r="B48" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C48" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -1214,10 +1217,10 @@
         <v>8</v>
       </c>
       <c r="B49" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C49" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -1225,10 +1228,10 @@
         <v>8</v>
       </c>
       <c r="B50" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C50" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -1236,10 +1239,10 @@
         <v>8</v>
       </c>
       <c r="B51" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C51" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -1247,10 +1250,10 @@
         <v>8</v>
       </c>
       <c r="B52" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C52" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -1258,10 +1261,10 @@
         <v>8</v>
       </c>
       <c r="B53" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C53" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -1269,10 +1272,10 @@
         <v>8</v>
       </c>
       <c r="B54" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C54" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -1280,10 +1283,10 @@
         <v>8</v>
       </c>
       <c r="B55" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C55" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -1291,10 +1294,10 @@
         <v>8</v>
       </c>
       <c r="B56" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C56" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -1302,10 +1305,10 @@
         <v>8</v>
       </c>
       <c r="B57" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C57" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1313,10 +1316,10 @@
         <v>8</v>
       </c>
       <c r="B58" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C58" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -1324,10 +1327,10 @@
         <v>9</v>
       </c>
       <c r="B59" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C59" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1335,10 +1338,10 @@
         <v>9</v>
       </c>
       <c r="B60" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C60" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1346,10 +1349,10 @@
         <v>9</v>
       </c>
       <c r="B61" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C61" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -1357,10 +1360,10 @@
         <v>9</v>
       </c>
       <c r="B62" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C62" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -1368,10 +1371,10 @@
         <v>9</v>
       </c>
       <c r="B63" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C63" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -1379,10 +1382,10 @@
         <v>9</v>
       </c>
       <c r="B64" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C64" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -1390,10 +1393,10 @@
         <v>9</v>
       </c>
       <c r="B65" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C65" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -1401,10 +1404,10 @@
         <v>9</v>
       </c>
       <c r="B66" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C66" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -1412,10 +1415,10 @@
         <v>9</v>
       </c>
       <c r="B67" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C67" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -1423,10 +1426,10 @@
         <v>10</v>
       </c>
       <c r="B68" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C68" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -1434,10 +1437,10 @@
         <v>10</v>
       </c>
       <c r="B69" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C69" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -1445,10 +1448,10 @@
         <v>10</v>
       </c>
       <c r="B70" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C70" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -1456,10 +1459,10 @@
         <v>10</v>
       </c>
       <c r="B71" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C71" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -1467,10 +1470,10 @@
         <v>10</v>
       </c>
       <c r="B72" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C72" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -1478,10 +1481,10 @@
         <v>10</v>
       </c>
       <c r="B73" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C73" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -1489,10 +1492,10 @@
         <v>10</v>
       </c>
       <c r="B74" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C74" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -1500,10 +1503,10 @@
         <v>10</v>
       </c>
       <c r="B75" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C75" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -1511,10 +1514,10 @@
         <v>11</v>
       </c>
       <c r="B76" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C76" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="77" spans="1:3">
@@ -1522,10 +1525,10 @@
         <v>11</v>
       </c>
       <c r="B77" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C77" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="78" spans="1:3">
@@ -1533,10 +1536,10 @@
         <v>11</v>
       </c>
       <c r="B78" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C78" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="79" spans="1:3">
@@ -1544,10 +1547,10 @@
         <v>11</v>
       </c>
       <c r="B79" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C79" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="80" spans="1:3">
@@ -1555,10 +1558,10 @@
         <v>11</v>
       </c>
       <c r="B80" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C80" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -1566,10 +1569,10 @@
         <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C81" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -1577,10 +1580,10 @@
         <v>11</v>
       </c>
       <c r="B82" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C82" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="83" spans="1:3">
@@ -1588,10 +1591,10 @@
         <v>11</v>
       </c>
       <c r="B83" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C83" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -1599,10 +1602,10 @@
         <v>12</v>
       </c>
       <c r="B84" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C84" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -1610,10 +1613,10 @@
         <v>12</v>
       </c>
       <c r="B85" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C85" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -1621,10 +1624,10 @@
         <v>12</v>
       </c>
       <c r="B86" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C86" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -1632,10 +1635,10 @@
         <v>12</v>
       </c>
       <c r="B87" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C87" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="88" spans="1:3">
@@ -1643,10 +1646,10 @@
         <v>12</v>
       </c>
       <c r="B88" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C88" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="89" spans="1:3">
@@ -1654,10 +1657,10 @@
         <v>12</v>
       </c>
       <c r="B89" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C89" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -1665,10 +1668,10 @@
         <v>13</v>
       </c>
       <c r="B90" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C90" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -1676,10 +1679,10 @@
         <v>13</v>
       </c>
       <c r="B91" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C91" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="92" spans="1:3">
@@ -1687,10 +1690,10 @@
         <v>13</v>
       </c>
       <c r="B92" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C92" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -1698,10 +1701,10 @@
         <v>13</v>
       </c>
       <c r="B93" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C93" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -1709,10 +1712,10 @@
         <v>13</v>
       </c>
       <c r="B94" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C94" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -1720,10 +1723,10 @@
         <v>13</v>
       </c>
       <c r="B95" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C95" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -1731,10 +1734,10 @@
         <v>13</v>
       </c>
       <c r="B96" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C96" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -1742,10 +1745,10 @@
         <v>14</v>
       </c>
       <c r="B97" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C97" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -1753,10 +1756,10 @@
         <v>14</v>
       </c>
       <c r="B98" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C98" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="99" spans="1:3">
@@ -1764,10 +1767,10 @@
         <v>14</v>
       </c>
       <c r="B99" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C99" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -1775,10 +1778,10 @@
         <v>14</v>
       </c>
       <c r="B100" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C100" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="101" spans="1:3">
@@ -1786,10 +1789,10 @@
         <v>14</v>
       </c>
       <c r="B101" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C101" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="102" spans="1:3">
@@ -1797,10 +1800,10 @@
         <v>14</v>
       </c>
       <c r="B102" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C102" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -1808,10 +1811,10 @@
         <v>14</v>
       </c>
       <c r="B103" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C103" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="104" spans="1:3">
@@ -1819,10 +1822,10 @@
         <v>14</v>
       </c>
       <c r="B104" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C104" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -1830,10 +1833,10 @@
         <v>15</v>
       </c>
       <c r="B105" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C105" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="106" spans="1:3">
@@ -1841,10 +1844,10 @@
         <v>15</v>
       </c>
       <c r="B106" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C106" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -1852,10 +1855,10 @@
         <v>15</v>
       </c>
       <c r="B107" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C107" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="108" spans="1:3">
@@ -1863,10 +1866,10 @@
         <v>15</v>
       </c>
       <c r="B108" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C108" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -1874,10 +1877,10 @@
         <v>15</v>
       </c>
       <c r="B109" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C109" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -1885,10 +1888,10 @@
         <v>15</v>
       </c>
       <c r="B110" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C110" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="111" spans="1:3">
@@ -1896,10 +1899,10 @@
         <v>15</v>
       </c>
       <c r="B111" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C111" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -1907,10 +1910,10 @@
         <v>15</v>
       </c>
       <c r="B112" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C112" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -1918,10 +1921,10 @@
         <v>15</v>
       </c>
       <c r="B113" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C113" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -1929,10 +1932,10 @@
         <v>16</v>
       </c>
       <c r="B114" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C114" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="115" spans="1:3">
@@ -1940,10 +1943,10 @@
         <v>16</v>
       </c>
       <c r="B115" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C115" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -1951,10 +1954,10 @@
         <v>16</v>
       </c>
       <c r="B116" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C116" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="117" spans="1:3">
@@ -1962,10 +1965,10 @@
         <v>16</v>
       </c>
       <c r="B117" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C117" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="118" spans="1:3">
@@ -1973,10 +1976,10 @@
         <v>16</v>
       </c>
       <c r="B118" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C118" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="119" spans="1:3">
@@ -1984,10 +1987,10 @@
         <v>4</v>
       </c>
       <c r="B119" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C119" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="120" spans="1:3">
@@ -1995,10 +1998,10 @@
         <v>4</v>
       </c>
       <c r="B120" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C120" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="121" spans="1:3">
@@ -2006,10 +2009,10 @@
         <v>4</v>
       </c>
       <c r="B121" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C121" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="122" spans="1:3">
@@ -2017,10 +2020,10 @@
         <v>5</v>
       </c>
       <c r="B122" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C122" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="123" spans="1:3">
@@ -2028,10 +2031,10 @@
         <v>5</v>
       </c>
       <c r="B123" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C123" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="124" spans="1:3">
@@ -2039,10 +2042,10 @@
         <v>5</v>
       </c>
       <c r="B124" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C124" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="125" spans="1:3">
@@ -2050,10 +2053,10 @@
         <v>5</v>
       </c>
       <c r="B125" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C125" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="126" spans="1:3">
@@ -2061,10 +2064,10 @@
         <v>7</v>
       </c>
       <c r="B126" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C126" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="127" spans="1:3">
@@ -2072,10 +2075,10 @@
         <v>7</v>
       </c>
       <c r="B127" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C127" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="128" spans="1:3">
@@ -2083,10 +2086,10 @@
         <v>8</v>
       </c>
       <c r="B128" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C128" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="129" spans="1:3">
@@ -2094,10 +2097,10 @@
         <v>8</v>
       </c>
       <c r="B129" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C129" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="130" spans="1:3">
@@ -2105,10 +2108,153 @@
         <v>10</v>
       </c>
       <c r="B130" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C130" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3">
+      <c r="A131" t="s">
+        <v>7</v>
+      </c>
+      <c r="B131" t="s">
+        <v>31</v>
+      </c>
+      <c r="C131" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3">
+      <c r="A132" t="s">
+        <v>7</v>
+      </c>
+      <c r="B132" t="s">
+        <v>30</v>
+      </c>
+      <c r="C132" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3">
+      <c r="A133" t="s">
+        <v>7</v>
+      </c>
+      <c r="B133" t="s">
+        <v>64</v>
+      </c>
+      <c r="C133" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3">
+      <c r="A134" t="s">
+        <v>7</v>
+      </c>
+      <c r="B134" t="s">
+        <v>72</v>
+      </c>
+      <c r="C134" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3">
+      <c r="A135" t="s">
+        <v>7</v>
+      </c>
+      <c r="B135" t="s">
+        <v>66</v>
+      </c>
+      <c r="C135" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3">
+      <c r="A136" t="s">
+        <v>17</v>
+      </c>
+      <c r="B136" t="s">
+        <v>104</v>
+      </c>
+      <c r="C136" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3">
+      <c r="A137" t="s">
+        <v>17</v>
+      </c>
+      <c r="B137" t="s">
+        <v>81</v>
+      </c>
+      <c r="C137" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3">
+      <c r="A138" t="s">
+        <v>17</v>
+      </c>
+      <c r="B138" t="s">
+        <v>105</v>
+      </c>
+      <c r="C138" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3">
+      <c r="A139" t="s">
+        <v>17</v>
+      </c>
+      <c r="B139" t="s">
+        <v>82</v>
+      </c>
+      <c r="C139" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3">
+      <c r="A140" t="s">
+        <v>17</v>
+      </c>
+      <c r="B140" t="s">
         <v>108</v>
+      </c>
+      <c r="C140" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3">
+      <c r="A141" t="s">
+        <v>17</v>
+      </c>
+      <c r="B141" t="s">
+        <v>69</v>
+      </c>
+      <c r="C141" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3">
+      <c r="A142" t="s">
+        <v>17</v>
+      </c>
+      <c r="B142" t="s">
+        <v>73</v>
+      </c>
+      <c r="C142" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3">
+      <c r="A143" t="s">
+        <v>17</v>
+      </c>
+      <c r="B143" t="s">
+        <v>55</v>
+      </c>
+      <c r="C143" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>